<commit_message>
1000 – 2025-01-09 14:54:35 – BR_README – TAMAR SAPIR – Create README.md file
</commit_message>
<xml_diff>
--- a/gitexcel.xlsx
+++ b/gitexcel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\סדנה מתקדמת בתוכנה לינוקס\Class8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1091623D-729C-4A11-B906-E30CF3808F72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{834218D5-D59E-4BD3-9645-989EB1768EB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CA8384D2-9D5E-4DB8-B7F3-3EC9EA562598}"/>
   </bookViews>
@@ -155,8 +155,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{83DF7497-33E1-487A-825F-CF1BFBAAF69D}" name="טבלה1" displayName="טבלה1" ref="A1:E1048576" totalsRowShown="0" dataDxfId="0">
-  <autoFilter ref="A1:E1048576" xr:uid="{83DF7497-33E1-487A-825F-CF1BFBAAF69D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{83DF7497-33E1-487A-825F-CF1BFBAAF69D}" name="טבלה1" displayName="טבלה1" ref="A1:E1037700" totalsRowShown="0" dataDxfId="0">
+  <autoFilter ref="A1:E1037700" xr:uid="{83DF7497-33E1-487A-825F-CF1BFBAAF69D}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{ADE1D384-CBB5-401A-A4DE-E6A80DE4D2B1}" name="TaskID" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{0C81459E-DC23-4682-9213-3748F2A9DBBF}" name="Desc" dataDxfId="4"/>

</xml_diff>